<commit_message>
Update stock bubble dashboard 2026-07-09 16:52:49
</commit_message>
<xml_diff>
--- a/stock_watch.xlsx
+++ b/stock_watch.xlsx
@@ -184,7 +184,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -296,7 +296,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -336,47 +336,47 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t/>
+          <t>2471.85</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t/>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t/>
+          <t>42.18%</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t/>
+          <t>-11.87%</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t/>
+          <t>-5.47%</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t/>
+          <t>-7.94%</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t/>
+          <t>61326.7亿</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>强势观察</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>中 / 波动30% / 回撤-21%</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -386,13 +386,12 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T3" t="str">
+        <f>HYPERLINK("kline_charts/BK0963_商业航天.html","打开K线图")</f>
+        <v>打开K线图</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -408,7 +407,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -520,7 +519,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -560,7 +559,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23.91</t>
+          <t>19.91</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -570,27 +569,27 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>144.73%</t>
+          <t>99.70%</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>9.58%</t>
+          <t>-31.44%</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>4.46%</t>
+          <t>-16.48%</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>-9.50%</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>1009.9亿</t>
+          <t>841.0亿</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -600,7 +599,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>高 / 波动60% / 回撤-40%</t>
+          <t>高 / 波动61% / 回撤-43%</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -631,7 +630,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -671,7 +670,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>167.00</t>
+          <t>148.05</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -681,27 +680,27 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>317.50%</t>
+          <t>274.15%</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>73.87%</t>
+          <t>33.11%</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>51.53%</t>
+          <t>21.82%</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>25.93%</t>
+          <t>8.26%</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>344.2亿</t>
+          <t>305.1亿</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -711,7 +710,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>高 / 波动56% / 回撤-37%</t>
+          <t>高 / 波动57% / 回撤-37%</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -742,7 +741,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -782,7 +781,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>32.76</t>
+          <t>32.81</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -792,27 +791,27 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>35.65%</t>
+          <t>33.54%</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2.06%</t>
+          <t>0.24%</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>35.76%</t>
+          <t>30.87%</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>26.19%</t>
+          <t>19.22%</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>125.5亿</t>
+          <t>125.7亿</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -853,7 +852,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -893,7 +892,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -903,27 +902,27 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>240.34%</t>
+          <t>253.81%</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>117.63%</t>
+          <t>103.97%</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>119.94%</t>
+          <t>110.53%</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>52.01%</t>
+          <t>45.75%</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>175.0亿</t>
+          <t>183.3亿</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -964,7 +963,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1004,7 +1003,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3.06</t>
+          <t>3.01</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1014,27 +1013,27 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>189.60%</t>
+          <t>184.23%</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>99.61%</t>
+          <t>97.90%</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>64.73%</t>
+          <t>51.48%</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>11.26%</t>
+          <t>2.24%</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>7600.0万</t>
+          <t>7400.0万</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1075,7 +1074,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1115,7 +1114,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>7.67</t>
+          <t>7.54</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1125,27 +1124,27 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>253.46%</t>
+          <t>242.97%</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>96.41%</t>
+          <t>95.03%</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>65.02%</t>
+          <t>50.48%</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>11.82%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>9600.0万</t>
+          <t>9300.0万</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1186,7 +1185,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1226,7 +1225,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>29.46</t>
+          <t>24.62</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1236,27 +1235,27 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>96.66%</t>
+          <t>68.28%</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>44.48%</t>
+          <t>22.61%</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>38.31%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>28.14%</t>
+          <t>4.10%</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>233.1亿</t>
+          <t>194.8亿</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1266,7 +1265,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>高 / 波动58% / 回撤-32%</t>
+          <t>高 / 波动60% / 回撤-32%</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1297,7 +1296,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1337,7 +1336,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>8722.84</t>
+          <t>8342.49</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1347,27 +1346,27 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>47.83%</t>
+          <t>39.44%</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>14.01%</t>
+          <t>5.67%</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>15.21%</t>
+          <t>5.62%</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>191015.4亿</t>
+          <t>182289.1亿</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1387,7 +1386,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t/>
+          <t>-</t>
         </is>
       </c>
       <c r="T12" t="str">
@@ -1408,7 +1407,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1448,7 +1447,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>41.21</t>
+          <t>37.69</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1458,27 +1457,27 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>80.98%</t>
+          <t>65.45%</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>11.41%</t>
+          <t>-13.36%</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>17.31%</t>
+          <t>-1.64%</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>24.28%</t>
+          <t>9.44%</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>135.1亿</t>
+          <t>123.5亿</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1519,7 +1518,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1559,7 +1558,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>40.00</t>
+          <t>36.19</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1569,27 +1568,27 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>245.01%</t>
+          <t>208.95%</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>207.13%</t>
+          <t>170.40%</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>122.05%</t>
+          <t>76.24%</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>-3.85%</t>
+          <t>-20.41%</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>274.8亿</t>
+          <t>248.6亿</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1599,7 +1598,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>高 / 波动69% / 回撤-23%</t>
+          <t>高 / 波动69% / 回撤-33%</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1630,7 +1629,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1670,7 +1669,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>10.92</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1680,27 +1679,27 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>110.00%</t>
+          <t>77.48%</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>48.37%</t>
+          <t>18.32%</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>40.90%</t>
+          <t>14.39%</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>32.52%</t>
+          <t>10.06%</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>550.4亿</t>
+          <t>468.8亿</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1710,7 +1709,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>高 / 波动52% / 回撤-33%</t>
+          <t>高 / 波动53% / 回撤-33%</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1741,7 +1740,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1781,7 +1780,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>106.77</t>
+          <t>93.56</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1791,27 +1790,27 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>452.35%</t>
+          <t>383.76%</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>245.20%</t>
+          <t>164.52%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>102.41%</t>
+          <t>68.33%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>35.79%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>697.3亿</t>
+          <t>611.1亿</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1821,7 +1820,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>高 / 波动71% / 回撤-23%</t>
+          <t>高 / 波动72% / 回撤-28%</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1852,7 +1851,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1892,7 +1891,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>62.30</t>
+          <t>55.77</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1902,27 +1901,27 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>129.57%</t>
+          <t>101.71%</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>74.67%</t>
+          <t>55.70%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>93.78%</t>
+          <t>64.51%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>-8.92%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>502.3亿</t>
+          <t>449.7亿</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -1932,7 +1931,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>高 / 波动51% / 回撤-25%</t>
+          <t>高 / 波动52% / 回撤-25%</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1963,7 +1962,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2003,7 +2002,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>696.55</t>
+          <t>600.99</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2013,27 +2012,27 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>754.57%</t>
+          <t>655.59%</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>146.68%</t>
+          <t>112.43%</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>134.92%</t>
+          <t>85.20%</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>43.60%</t>
+          <t>16.78%</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2946.8亿</t>
+          <t>2542.6亿</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2074,7 +2073,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2186,7 +2185,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2226,7 +2225,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>55.43</t>
+          <t>50.54</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2236,27 +2235,27 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>206.92%</t>
+          <t>175.87%</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>203.73%</t>
+          <t>161.46%</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>156.38%</t>
+          <t>120.60%</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>29.57%</t>
+          <t>11.37%</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>213.8亿</t>
+          <t>194.9亿</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2266,7 +2265,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>高 / 波动51% / 回撤-32%</t>
+          <t>高 / 波动53% / 回撤-32%</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2297,7 +2296,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2337,7 +2336,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>28.50</t>
+          <t>25.14</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2347,27 +2346,27 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>343.58%</t>
+          <t>277.19%</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>246.08%</t>
+          <t>198.75%</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>225.90%</t>
+          <t>162.83%</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>91.60%</t>
+          <t>61.72%</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>596.1亿</t>
+          <t>525.8亿</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2377,17 +2376,17 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>高 / 波动62% / 回撤-27%</t>
+          <t>高 / 波动64% / 回撤-27%</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>化学纤维及制品、化纤产品、化纤机械及配件、纺织机械及配件、通用设备、电机、汽车零配件的制造、加工;机械设备的安装、维修服务;纺织技术服务;化纤的工艺设计、开发;针纺织品、纺织原料(不含棉花、蚕茧)的制造、加工、销售;化工原料(不含危险化学品)、仪器仪表、电子产品及通信设备(地面卫星接收设施外)、建筑用材料、塑料制品、金属材料的销售;自营和代理各类商品及技术的进出口业务(国家限定企业经营或禁止进出口的商品和技术除外);机械设备租赁(不含…</t>
+          <t/>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>建筑-建筑施工-专业工程</t>
+          <t/>
         </is>
       </c>
       <c r="T21" t="str">
@@ -2408,7 +2407,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2448,7 +2447,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>126.00</t>
+          <t>118.22</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2458,27 +2457,27 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>401.19%</t>
+          <t>392.99%</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>267.13%</t>
+          <t>221.16%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>282.98%</t>
+          <t>201.43%</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>-7.69%</t>
+          <t>-21.27%</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>283.2亿</t>
+          <t>265.7亿</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2488,7 +2487,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>高 / 波动74% / 回撤-31%</t>
+          <t>高 / 波动74% / 回撤-34%</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2519,7 +2518,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2559,7 +2558,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>332.00</t>
+          <t>337.13</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2569,27 +2568,27 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>364.23%</t>
+          <t>364.39%</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>232.28%</t>
+          <t>201.29%</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>122.63%</t>
+          <t>115.30%</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>71.51%</t>
+          <t>49.92%</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>916.2亿</t>
+          <t>930.4亿</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2604,12 +2603,12 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t/>
+          <t>一般项目:电子专用材料研发;电子专用材料制造;电子专用材料销售;电子元器件制造;电子元器件零售;电子专用设备制造;电子专用设备销售;有色金属压延加工;常用有色金属冶炼;有色金属铸造;金属材料制造;新材料技术研发;软件开发;信息系统集成服务;智能控制系统集成;物联网应用服务;物联网技术服务;人工智能基础资源与技术平台(除依法须经批准的项目外,凭营业执照依法自主开展经营活动)。许可项目:检验检测服务;技术进出口;进出口代理;货物进出口(依…</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t/>
+          <t>电子设备-半导体-半导体材料</t>
         </is>
       </c>
       <c r="T23" t="str">
@@ -2630,7 +2629,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2670,7 +2669,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>47.54</t>
+          <t>40.98</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2680,27 +2679,27 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>307.68%</t>
+          <t>242.18%</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>36.62%</t>
+          <t>25.30%</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>74.81%</t>
+          <t>50.08%</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>41.36%</t>
+          <t>20.74%</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>565.9亿</t>
+          <t>487.8亿</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2710,7 +2709,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>高 / 波动65% / 回撤-37%</t>
+          <t>高 / 波动66% / 回撤-37%</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2741,7 +2740,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2781,7 +2780,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>24.35</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2791,27 +2790,27 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>106.36%</t>
+          <t>47.93%</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>-6.63%</t>
+          <t>-19.78%</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>-13.16%</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>5.27%</t>
+          <t>-12.74%</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>225.3亿</t>
+          <t>185.0亿</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2821,7 +2820,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>高 / 波动63% / 回撤-33%</t>
+          <t>高 / 波动64% / 回撤-36%</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2852,7 +2851,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2964,7 +2963,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3004,7 +3003,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>235.19</t>
+          <t>196.00</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3014,27 +3013,27 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>126.47%</t>
+          <t>86.58%</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>49.57%</t>
+          <t>28.78%</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>36.14%</t>
+          <t>8.88%</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>28.39%</t>
+          <t>7.05%</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>673.4亿</t>
+          <t>561.2亿</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3044,7 +3043,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>高 / 波动50% / 回撤-25%</t>
+          <t>高 / 波动51% / 回撤-25%</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -3075,7 +3074,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3115,7 +3114,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>129.83</t>
+          <t>107.90</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -3125,27 +3124,27 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>467.19%</t>
+          <t>315.58%</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>57.04%</t>
+          <t>23.97%</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>70.17%</t>
+          <t>33.78%</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>8.64%</t>
+          <t>-8.44%</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>153.8亿</t>
+          <t>127.8亿</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -3186,7 +3185,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3226,7 +3225,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>92.07</t>
+          <t>80.16</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3236,27 +3235,27 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>89.76%</t>
+          <t>67.38%</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>78.15%</t>
+          <t>27.26%</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>37.99%</t>
+          <t>2.48%</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>54.27%</t>
+          <t>30.64%</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>418.0亿</t>
+          <t>363.9亿</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3266,7 +3265,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>高 / 波动56% / 回撤-30%</t>
+          <t>高 / 波动57% / 回撤-30%</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -3297,7 +3296,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3337,7 +3336,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>211.06</t>
+          <t>199.00</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -3347,27 +3346,27 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>305.11%</t>
+          <t>277.82%</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>105.31%</t>
+          <t>90.52%</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>80.79%</t>
+          <t>56.93%</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>70.48%</t>
+          <t>54.29%</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>988.3亿</t>
+          <t>931.8亿</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -3377,7 +3376,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>高 / 波动77% / 回撤-34%</t>
+          <t>高 / 波动76% / 回撤-34%</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3408,7 +3407,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3520,7 +3519,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3560,7 +3559,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>44.32</t>
+          <t>34.74</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3570,27 +3569,27 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>605.73%</t>
+          <t>423.98%</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>431.41%</t>
+          <t>312.10%</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>64.82%</t>
+          <t>31.79%</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>12.77%</t>
+          <t>-15.78%</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>306.4亿</t>
+          <t>240.2亿</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -3600,7 +3599,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>高 / 波动75% / 回撤-37%</t>
+          <t>高 / 波动77% / 回撤-39%</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3631,7 +3630,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3671,7 +3670,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>6.37</t>
+          <t>4.72</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3681,37 +3680,37 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>7.24%</t>
+          <t>-26.13%</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>-12.14%</t>
+          <t>-36.81%</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>17.96%</t>
+          <t>-10.61%</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>64.18%</t>
+          <t>21.03%</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>82.6亿</t>
+          <t>61.2亿</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>谨慎</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>高 / 波动57% / 回撤-58%</t>
+          <t>高 / 波动59% / 回撤-58%</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3742,7 +3741,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3782,7 +3781,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>74.41</t>
+          <t>64.05</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3792,27 +3791,27 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>213.27%</t>
+          <t>158.86%</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>52.07%</t>
+          <t>32.93%</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>59.16%</t>
+          <t>24.87%</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>44.65%</t>
+          <t>17.93%</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>222.9亿</t>
+          <t>191.8亿</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -3822,7 +3821,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>高 / 波动68% / 回撤-23%</t>
+          <t>高 / 波动69% / 回撤-23%</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3853,7 +3852,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3893,7 +3892,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>129.05</t>
+          <t>113.72</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3903,27 +3902,27 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>383.71%</t>
+          <t>323.54%</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>174.78%</t>
+          <t>135.10%</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>105.17%</t>
+          <t>53.01%</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>40.98%</t>
+          <t>9.35%</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>483.0亿</t>
+          <t>425.6亿</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3964,7 +3963,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4004,7 +4003,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4014,27 +4013,27 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>213.69%</t>
+          <t>186.84%</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>88.74%</t>
+          <t>77.80%</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>97.02%</t>
+          <t>76.17%</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>38.30%</t>
+          <t>23.27%</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2.1亿</t>
+          <t>1.7亿</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -4044,7 +4043,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>高 / 波动45% / 回撤-17%</t>
+          <t>高 / 波动45% / 回撤-21%</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -4054,7 +4053,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>-</t>
+          <t/>
         </is>
       </c>
       <c r="T36" t="str">
@@ -4075,7 +4074,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4115,7 +4114,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1116.99</t>
+          <t>1146.00</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -4125,27 +4124,27 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>735.13%</t>
+          <t>689.31%</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>79.43%</t>
+          <t>92.78%</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>80.59%</t>
+          <t>65.60%</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-2.88%</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>12457.1亿</t>
+          <t>12780.6亿</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -4155,7 +4154,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>高 / 波动72% / 回撤-21%</t>
+          <t>高 / 波动71% / 回撤-21%</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -4186,7 +4185,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4226,7 +4225,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>521.72</t>
+          <t>520.96</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -4236,27 +4235,27 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>482.04%</t>
+          <t>452.32%</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>71.61%</t>
+          <t>78.18%</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>59.58%</t>
+          <t>49.15%</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>0.89%</t>
+          <t>-7.06%</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>7274.1亿</t>
+          <t>7263.5亿</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -4297,7 +4296,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4337,7 +4336,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>671.03</t>
+          <t>640.00</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4347,27 +4346,27 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>458.91%</t>
+          <t>445.56%</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>185.63%</t>
+          <t>148.06%</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>169.59%</t>
+          <t>156.27%</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>41.56%</t>
+          <t>27.87%</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>4708.9亿</t>
+          <t>4491.2亿</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -4377,7 +4376,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>高 / 波动67% / 回撤-28%</t>
+          <t>高 / 波动68% / 回撤-28%</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4408,7 +4407,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4448,7 +4447,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>148.29</t>
+          <t>142.50</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -4458,27 +4457,27 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>184.79%</t>
+          <t>172.21%</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>71.14%</t>
+          <t>20.09%</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>65.71%</t>
+          <t>48.47%</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>45.38%</t>
+          <t>26.11%</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>646.5亿</t>
+          <t>621.3亿</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -4519,7 +4518,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4559,7 +4558,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>133.92</t>
+          <t>124.71</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4569,27 +4568,27 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>464.82%</t>
+          <t>413.21%</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>215.03%</t>
+          <t>193.64%</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>108.73%</t>
+          <t>63.75%</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>10.81%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>1378.8亿</t>
+          <t>1284.0亿</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -4630,7 +4629,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4670,7 +4669,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>3.22</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -4680,27 +4679,27 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>-2.72%</t>
+          <t>-11.50%</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>9.15%</t>
+          <t>2.04%</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>29.84%</t>
+          <t>9.49%</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>-43.80%</t>
+          <t>-47.37%</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>68.3亿</t>
+          <t>63.6亿</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -4710,17 +4709,17 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>高 / 波动55% / 回撤-44%</t>
+          <t>高 / 波动55% / 回撤-48%</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>一般经营项目是:互联网、云计算软件与平台服务;物联网系统研发与应用服务;智慧医疗信息系统研发与集成服务;医疗大数据开发与应用服务;医疗专业系统咨询、设计、集成服务;医疗投资管理;智能交通含轨道交通信号监控系统开发、技术咨询设计、销售与集成服务;智能建筑系统开发与集成、技术咨询设计;机电总包服务;智能卡、智能管控、安防监控等终端设备与软件的研发、销售及应用服务;能源监测与节能服务;合同能源管理服务;新能源技术开发和咨询设计服务;电力销售…</t>
+          <t/>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>信息技术-计算机软件-行业应用软件</t>
+          <t/>
         </is>
       </c>
       <c r="T42" t="str">
@@ -4741,7 +4740,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4781,7 +4780,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>103.64</t>
+          <t>95.20</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4791,27 +4790,27 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>358.36%</t>
+          <t>264.88%</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>40.05%</t>
+          <t>36.08%</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>88.33%</t>
+          <t>46.01%</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>-7.57%</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>243.2亿</t>
+          <t>223.4亿</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -4852,7 +4851,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4892,7 +4891,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>90.91</t>
+          <t>92.27</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4902,27 +4901,27 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>219.77%</t>
+          <t>226.97%</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>133.34%</t>
+          <t>103.06%</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>84.03%</t>
+          <t>76.59%</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>40.27%</t>
+          <t>33.72%</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>866.6亿</t>
+          <t>879.6亿</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -4963,7 +4962,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5003,7 +5002,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>112.42</t>
+          <t>96.67</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -5013,27 +5012,27 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>344.98%</t>
+          <t>281.24%</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>-21.65%</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>12.29%</t>
+          <t>-9.71%</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>15.08%</t>
+          <t>-3.19%</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>211.3亿</t>
+          <t>181.7亿</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -5074,7 +5073,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5114,7 +5113,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>18.54</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -5124,27 +5123,27 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>101.78%</t>
+          <t>96.56%</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>16.93%</t>
+          <t>-0.44%</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>35.69%</t>
+          <t>27.51%</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>34.35%</t>
+          <t>20.69%</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>208.9亿</t>
+          <t>203.7亿</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -5185,7 +5184,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5225,7 +5224,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>45.45</t>
+          <t>40.88</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -5235,27 +5234,27 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>242.24%</t>
+          <t>190.13%</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>172.32%</t>
+          <t>131.61%</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>228.87%</t>
+          <t>176.96%</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>85.13%</t>
+          <t>56.69%</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>376.7亿</t>
+          <t>338.8亿</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -5265,7 +5264,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>高 / 波动67% / 回撤-34%</t>
+          <t>高 / 波动68% / 回撤-34%</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -5296,7 +5295,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5336,7 +5335,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5346,27 +5345,27 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>-33.96%</t>
+          <t>-37.82%</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>-19.35%</t>
+          <t>-23.32%</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>19.86%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>-9.79%</t>
+          <t>-9.52%</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>48.6亿</t>
+          <t>47.4亿</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5376,17 +5375,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>高 / 波动53% / 回撤-51%</t>
+          <t>高 / 波动54% / 回撤-51%</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t/>
+          <t>制作、复制、发行:专题、专栏、综艺、动画片、广播剧、电视剧(凭节目制作经营许可证在核定期限内经营);企业形象策划;影视文化信息咨询服务;影视广告制作、代理、发布;国产影片发行(凭电影发行经营许可证在核定期限内经营);摄制电影(单片);影视项目的投资管理;经营进出口业务(国家法律法规禁止、限制的除外);股权投资,项目投资;投资管理;资产管理;投资咨询;企业管理咨询;经济贸易咨询;企业形象策划。</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>影视院线</t>
+          <t>文化传媒-影视动漫-影视</t>
         </is>
       </c>
       <c r="T48" t="str">
@@ -5407,7 +5406,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5447,47 +5446,47 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>3299.09</t>
+          <t/>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t/>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>137.58%</t>
+          <t/>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>79.31%</t>
+          <t/>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>62.86%</t>
+          <t/>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>5.10%</t>
+          <t/>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>17054.1亿</t>
+          <t/>
         </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>强势观察</t>
+          <t>待评估</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>中 / 波动33% / 回撤-14%</t>
+          <t>待评估</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -5497,12 +5496,13 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T49" t="str">
-        <f>HYPERLINK("kline_charts/BK1175_玻璃基板.html","打开K线图")</f>
-        <v>打开K线图</v>
+          <t/>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
@@ -5518,7 +5518,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>24.06</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5568,27 +5568,27 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>114.06%</t>
+          <t>95.48%</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>98.84%</t>
+          <t>63.12%</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>94.35%</t>
+          <t>72.29%</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>9.36%</t>
+          <t>-2.73%</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>227.3亿</t>
+          <t>208.5亿</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>高 / 波动53% / 回撤-26%</t>
+          <t>高 / 波动53% / 回撤-33%</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -5629,7 +5629,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5669,7 +5669,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>27.47</t>
+          <t>24.77</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -5679,27 +5679,27 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>49.70%</t>
+          <t>36.40%</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>-0.07%</t>
+          <t>-8.83%</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>-8.52%</t>
+          <t>-21.81%</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>1.93%</t>
+          <t>-11.25%</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>589.0亿</t>
+          <t>531.1亿</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>高 / 波动47% / 回撤-30%</t>
+          <t>高 / 波动48% / 回撤-34%</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -5740,7 +5740,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -5852,7 +5852,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>24.51</t>
+          <t>22.51</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -5902,27 +5902,27 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>22.86%</t>
+          <t>11.88%</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>22.12%</t>
+          <t>2.23%</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>14.00%</t>
+          <t>-9.96%</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>17.05%</t>
+          <t>4.21%</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>61.7亿</t>
+          <t>56.7亿</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -5963,7 +5963,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6003,7 +6003,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>481.00</t>
+          <t>394.92</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -6013,27 +6013,27 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>317.82%</t>
+          <t>232.26%</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>151.75%</t>
+          <t>106.76%</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>159.08%</t>
+          <t>98.17%</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>12.32%</t>
+          <t>-6.01%</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>881.8亿</t>
+          <t>724.0亿</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6043,7 +6043,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>高 / 波动65% / 回撤-25%</t>
+          <t>高 / 波动67% / 回撤-25%</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -6074,7 +6074,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>113.21</t>
+          <t>86.29</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -6124,27 +6124,27 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>440.98%</t>
+          <t>308.43%</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>86.94%</t>
+          <t>42.16%</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>116.84%</t>
+          <t>62.44%</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>30.11%</t>
+          <t>-0.35%</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>348.9亿</t>
+          <t>266.0亿</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>高 / 波动74% / 回撤-35%</t>
+          <t>高 / 波动75% / 回撤-35%</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -6185,7 +6185,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6225,7 +6225,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>41.91</t>
+          <t>34.20</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -6235,27 +6235,27 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>-8.47%</t>
+          <t>-23.47%</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>-15.91%</t>
+          <t>-34.93%</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>-34.87%</t>
+          <t>-45.12%</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>34.24%</t>
+          <t>8.67%</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>467.2亿</t>
+          <t>381.3亿</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -6296,7 +6296,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6336,7 +6336,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>87.64</t>
+          <t>89.38</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -6346,27 +6346,27 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>175.16%</t>
+          <t>182.31%</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>50.84%</t>
+          <t>49.64%</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>89.37%</t>
+          <t>83.34%</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>42.32%</t>
+          <t>20.95%</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>357.4亿</t>
+          <t>364.5亿</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
@@ -6381,12 +6381,12 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>压力管道组件、各类低功率气动控制阀、流体设备、真空电子洁净设备及其相关零配件、精密模具的加工、制造;航空、航天、汽车、摩托车轻量化及环保型新材料研发与制造;新能源发电成套设备或关键设备制造;并销售自产产品,提供售后服务。本公司同类产品的批发、进出口、佣金代理(拍卖除外)及技术服务等;道路普通货物运输。(上述涉及配额、许可证管理及专项管理的商品,根据国家有关规定办理)(依法须经批准的项目,经相关部门批准后方可开展经营活动)。</t>
+          <t/>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>机械设备-通用设备-基础件</t>
+          <t/>
         </is>
       </c>
       <c r="T57" t="str">
@@ -6407,7 +6407,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>193.17</t>
+          <t>170.99</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -6457,27 +6457,27 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>511.99%</t>
+          <t>431.72%</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>135.91%</t>
+          <t>101.10%</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>106.48%</t>
+          <t>67.04%</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>37.68%</t>
+          <t>17.54%</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>243.1亿</t>
+          <t>215.2亿</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -6518,7 +6518,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>181.50</t>
+          <t>183.44</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -6568,27 +6568,27 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>216.75%</t>
+          <t>227.05%</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>64.39%</t>
+          <t>62.55%</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>28.86%</t>
+          <t>20.64%</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>31.03%</t>
+          <t>26.64%</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>305.1亿</t>
+          <t>308.3亿</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -6629,7 +6629,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -6669,7 +6669,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>304.08</t>
+          <t>317.50</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -6679,27 +6679,27 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>580.73%</t>
+          <t>627.21%</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>187.14%</t>
+          <t>156.98%</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>155.79%</t>
+          <t>136.76%</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>51.74%</t>
+          <t>49.25%</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>1929.1亿</t>
+          <t>2014.3亿</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -6740,7 +6740,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>199.82</t>
+          <t>216.02</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -6790,27 +6790,27 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>251.46%</t>
+          <t>288.49%</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>93.44%</t>
+          <t>90.76%</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>111.03%</t>
+          <t>110.14%</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>61.93%</t>
+          <t>65.08%</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>335.7亿</t>
+          <t>362.9亿</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>高 / 波动65% / 回撤-30%</t>
+          <t>高 / 波动66% / 回撤-30%</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -6851,7 +6851,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -6891,7 +6891,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>252.36</t>
+          <t>263.04</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -6901,27 +6901,27 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>382.15%</t>
+          <t>407.30%</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>263.06%</t>
+          <t>225.14%</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>178.14%</t>
+          <t>171.51%</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>83.99%</t>
+          <t>59.82%</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>772.8亿</t>
+          <t>805.5亿</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -6962,7 +6962,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -7074,7 +7074,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>86.06</t>
+          <t>84.94</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -7124,27 +7124,27 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>175.29%</t>
+          <t>171.36%</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>92.09%</t>
+          <t>51.05%</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>76.85%</t>
+          <t>66.02%</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>65.63%</t>
+          <t>51.52%</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>530.2亿</t>
+          <t>523.3亿</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -7154,7 +7154,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>高 / 波动53% / 回撤-26%</t>
+          <t>高 / 波动54% / 回撤-26%</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -7185,7 +7185,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -7225,7 +7225,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>187.86</t>
+          <t>199.00</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -7235,27 +7235,27 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>260.02%</t>
+          <t>275.76%</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>142.53%</t>
+          <t>131.64%</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>140.45%</t>
+          <t>136.51%</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>77.86%</t>
+          <t>78.62%</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>894.1亿</t>
+          <t>947.1亿</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -7270,12 +7270,12 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t/>
+          <t>许可项目:危险化学品生产(依法须经批准的项目,经相关部门批准后方可开展经营活动,具体经营项目以审批结果为准)一般项目:新材料技术研发;专用化学产品制造(不含危险化学品);专用化学产品销售(不含危险化学品);纸和纸板容器制造;塑料包装箱及容器制造;玻璃纤维增强塑料制品制造;玻璃纤维增强塑料制品销售;塑料制品制造;塑料制品销售;工程和技术研究和试验发展;自然科学研究和试验发展;技术服务、技术开发、技术咨询、技术交流、技术转让、技术推广;货…</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t/>
+          <t>电子设备-半导体-半导体材料</t>
         </is>
       </c>
       <c r="T65" t="str">
@@ -7296,7 +7296,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -7336,7 +7336,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>225.33</t>
+          <t>204.35</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -7346,27 +7346,27 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>1016.49%</t>
+          <t>830.47%</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>494.82%</t>
+          <t>445.92%</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>226.89%</t>
+          <t>168.42%</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>19.54%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2038.3亿</t>
+          <t>1848.5亿</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -7381,12 +7381,12 @@
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>一般项目:货物进出口;技术进出口;玻璃纤维及制品制造;玻璃纤维及制品销售;电子专用材料制造;电子专用材料销售;电子专用材料研发;合成材料制造(不含危险化学品);合成材料销售;新材料技术研发;高性能纤维及复合材料制造;高性能纤维及复合材料销售;化工产品销售(不含许可类化工产品);电子专用设备销售;纺织专用设备销售。技术服务、技术开发、技术咨询、技术交流、技术转让、技术推广。(除依法须经批准的项目外,凭营业执照依法自主开展经营活动)。</t>
+          <t/>
         </is>
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>基础化工-合成纤维及树脂-玻纤</t>
+          <t/>
         </is>
       </c>
       <c r="T66" t="str">
@@ -7407,7 +7407,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -7447,7 +7447,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>65.24</t>
+          <t>54.58</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -7457,27 +7457,27 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>458.56%</t>
+          <t>356.74%</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>276.89%</t>
+          <t>214.40%</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>149.58%</t>
+          <t>96.26%</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>83.46%</t>
+          <t>39.52%</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2611.7亿</t>
+          <t>2184.9亿</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -7487,7 +7487,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>高 / 波动56% / 回撤-21%</t>
+          <t>高 / 波动57% / 回撤-26%</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -7518,7 +7518,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>77.84</t>
+          <t>70.77</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -7568,27 +7568,27 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>246.63%</t>
+          <t>192.12%</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>107.32%</t>
+          <t>93.91%</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>93.46%</t>
+          <t>65.91%</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>32.38%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>1306.2亿</t>
+          <t>1187.6亿</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -7598,17 +7598,17 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>高 / 波动71% / 回撤-26%</t>
+          <t>高 / 波动72% / 回撤-28%</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>一般项目:新材料技术研发;玻璃纤维及制品制造;玻璃纤维及制品销售;高性能纤维及复合材料制造;高性能纤维及复合材料销售;隔热和隔音材料制造;隔热和隔音材料销售;有色金属压延加工;专用化学产品制造(不含危险化学品);专用化学产品销售(不含危险化学品);技术服务、技术开发、技术咨询、技术交流、技术转让、技术推广;工业工程设计服务;对外承包工程;特种设备销售;有色金属合金销售;机械设备销售;工业自动控制系统装置销售;工业控制计算机及系统销售;…</t>
+          <t/>
         </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>基础化工-合成纤维及树脂-玻纤</t>
+          <t/>
         </is>
       </c>
       <c r="T68" t="str">
@@ -7629,7 +7629,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -7669,7 +7669,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>41.84</t>
+          <t>36.55</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -7679,27 +7679,27 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>900.96%</t>
+          <t>566.97%</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>484.36%</t>
+          <t>406.93%</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>266.05%</t>
+          <t>192.40%</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>90.53%</t>
+          <t>44.24%</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>1577.7亿</t>
+          <t>1378.3亿</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -7709,7 +7709,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>高 / 波动89% / 回撤-35%</t>
+          <t>高 / 波动90% / 回撤-35%</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -7740,7 +7740,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -7852,7 +7852,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>21.27</t>
+          <t>22.00</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -7902,27 +7902,27 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>5.98%</t>
+          <t>4.52%</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>-13.74%</t>
+          <t>-8.86%</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>-11.22%</t>
+          <t>-4.96%</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>4.52%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>111.8亿</t>
+          <t>115.6亿</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -7932,7 +7932,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>高 / 波动43% / 回撤-38%</t>
+          <t>高 / 波动42% / 回撤-38%</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -7963,7 +7963,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>8.65</t>
+          <t>7.70</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -8013,37 +8013,37 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>27.02%</t>
+          <t>9.84%</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>19.64%</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>29.30%</t>
+          <t>13.57%</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>11.61%</t>
+          <t>-9.73%</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>37.4亿</t>
+          <t>33.3亿</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>强势观察</t>
+          <t>偏强</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>中 / 波动45% / 回撤-26%</t>
+          <t>高 / 波动45% / 回撤-26%</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -8074,7 +8074,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>8.35</t>
+          <t>7.65</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -8124,27 +8124,27 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>20.49%</t>
+          <t>10.55%</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>-24.30%</t>
+          <t>-40.05%</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>-13.11%</t>
+          <t>-23.58%</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>-0.24%</t>
+          <t>-7.50%</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>58.9亿</t>
+          <t>53.9亿</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -8185,7 +8185,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -8225,7 +8225,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>7.49</t>
+          <t>7.66</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -8235,27 +8235,27 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>-20.91%</t>
+          <t>-19.71%</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>-18.76%</t>
+          <t>-19.28%</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>-0.27%</t>
+          <t>-1.29%</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>6.83%</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>110.8亿</t>
+          <t>113.3亿</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -8265,7 +8265,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>高 / 波动39% / 回撤-43%</t>
+          <t>高 / 波动40% / 回撤-42%</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -8296,7 +8296,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>2.67</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -8346,27 +8346,27 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>-33.90%</t>
+          <t>-39.59%</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>-31.20%</t>
+          <t>-34.72%</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>-22.87%</t>
+          <t>-26.85%</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>-7.28%</t>
+          <t>-11.88%</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>44.9亿</t>
+          <t>42.8亿</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
@@ -8376,7 +8376,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>高 / 波动30% / 回撤-43%</t>
+          <t>高 / 波动30% / 回撤-44%</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -8407,7 +8407,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -8447,7 +8447,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>9.35</t>
+          <t>7.82</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -8457,27 +8457,27 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>175.00%</t>
+          <t>127.99%</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>135.52%</t>
+          <t>89.81%</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>167.14%</t>
+          <t>120.28%</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>47.24%</t>
+          <t>26.74%</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>104.4亿</t>
+          <t>87.3亿</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
@@ -8487,7 +8487,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>高 / 波动51% / 回撤-26%</t>
+          <t>高 / 波动52% / 回撤-26%</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -8518,7 +8518,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>34.70</t>
+          <t>30.62</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -8568,27 +8568,27 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>20.71%</t>
+          <t>12.59%</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>-43.69%</t>
+          <t>-52.32%</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>-14.24%</t>
+          <t>-29.00%</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>-8.52%</t>
+          <t>-18.78%</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>87.4亿</t>
+          <t>77.2亿</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -8598,7 +8598,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>高 / 波动73% / 回撤-53%</t>
+          <t>高 / 波动73% / 回撤-55%</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -8629,7 +8629,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>21.26</t>
+          <t>19.34</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -8679,27 +8679,27 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>31.31%</t>
+          <t>19.45%</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>-9.15%</t>
+          <t>-19.82%</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>4.98%</t>
+          <t>-8.08%</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>-7.33%</t>
+          <t>-17.14%</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>83.4亿</t>
+          <t>75.9亿</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -8709,7 +8709,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>高 / 波动51% / 回撤-35%</t>
+          <t>高 / 波动50% / 回撤-35%</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -8740,7 +8740,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-06 12:59</t>
+          <t>2026-07-09 12:26</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>43.59</t>
+          <t>42.88</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -8790,27 +8790,27 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>-10.27%</t>
+          <t>-6.92%</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>-18.34%</t>
+          <t>-21.47%</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>-8.19%</t>
+          <t>-10.94%</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>-23.34%</t>
+          <t>-25.24%</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>37.3亿</t>
+          <t>36.7亿</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -14126,7 +14126,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>52.01%</t>
+          <t>45.75%</t>
         </is>
       </c>
       <c r="J4" t="str">
@@ -14182,7 +14182,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>61.93%</t>
+          <t>65.08%</t>
         </is>
       </c>
       <c r="J5" t="str">
@@ -14238,7 +14238,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>31.03%</t>
+          <t>26.64%</t>
         </is>
       </c>
       <c r="J6" t="str">
@@ -14294,7 +14294,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>91.60%</t>
+          <t>61.72%</t>
         </is>
       </c>
       <c r="J7" t="str">
@@ -14350,7 +14350,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>83.99%</t>
+          <t>59.82%</t>
         </is>
       </c>
       <c r="J8" t="str">
@@ -14406,7 +14406,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>42.32%</t>
+          <t>20.95%</t>
         </is>
       </c>
       <c r="J9" t="str">
@@ -14462,7 +14462,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>71.51%</t>
+          <t>49.92%</t>
         </is>
       </c>
       <c r="J10" t="str">
@@ -14518,7 +14518,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>29.57%</t>
+          <t>11.37%</t>
         </is>
       </c>
       <c r="J11" t="str">
@@ -14574,7 +14574,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>-7.69%</t>
+          <t>-21.27%</t>
         </is>
       </c>
       <c r="J12" t="str">
@@ -14630,7 +14630,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>45.38%</t>
+          <t>26.11%</t>
         </is>
       </c>
       <c r="J13" t="str">
@@ -14686,7 +14686,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>26.19%</t>
+          <t>19.22%</t>
         </is>
       </c>
       <c r="J14" t="str">
@@ -14742,7 +14742,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>51.74%</t>
+          <t>49.25%</t>
         </is>
       </c>
       <c r="J15" t="str">
@@ -14798,7 +14798,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>40.27%</t>
+          <t>33.72%</t>
         </is>
       </c>
       <c r="J16" t="str">
@@ -14968,7 +14968,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-0.24%</t>
+          <t>-7.50%</t>
         </is>
       </c>
       <c r="J19" t="str">
@@ -15024,7 +15024,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>-23.34%</t>
+          <t>-25.24%</t>
         </is>
       </c>
       <c r="J20" t="str">
@@ -15080,7 +15080,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-8.52%</t>
+          <t>-18.78%</t>
         </is>
       </c>
       <c r="J21" t="str">
@@ -15136,7 +15136,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>47.24%</t>
+          <t>26.74%</t>
         </is>
       </c>
       <c r="J22" t="str">
@@ -15192,7 +15192,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>11.61%</t>
+          <t>-9.73%</t>
         </is>
       </c>
       <c r="J23" t="str">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>6.83%</t>
         </is>
       </c>
       <c r="J24" t="str">
@@ -15304,7 +15304,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>-7.33%</t>
+          <t>-17.14%</t>
         </is>
       </c>
       <c r="J25" t="str">
@@ -15360,7 +15360,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>4.52%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="J26" t="str">
@@ -15416,7 +15416,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>-7.28%</t>
+          <t>-11.88%</t>
         </is>
       </c>
       <c r="J27" t="str">
@@ -15529,12 +15529,13 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>5.10%</t>
-        </is>
-      </c>
-      <c r="J29" t="str">
-        <f>HYPERLINK("kline_charts/BK1175_玻璃基板.html","打开K线图")</f>
-        <v>打开K线图</v>
+          <t/>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -15642,7 +15643,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>83.46%</t>
+          <t>39.52%</t>
         </is>
       </c>
       <c r="J31" t="str">
@@ -15698,7 +15699,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>32.38%</t>
+          <t>9.42%</t>
         </is>
       </c>
       <c r="J32" t="str">
@@ -15754,7 +15755,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>9.36%</t>
+          <t>-2.73%</t>
         </is>
       </c>
       <c r="J33" t="str">
@@ -15810,7 +15811,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>90.53%</t>
+          <t>44.24%</t>
         </is>
       </c>
       <c r="J34" t="str">
@@ -15866,7 +15867,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>19.54%</t>
+          <t>-1.44%</t>
         </is>
       </c>
       <c r="J35" t="str">
@@ -15922,7 +15923,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>17.05%</t>
+          <t>4.21%</t>
         </is>
       </c>
       <c r="J36" t="str">
@@ -16092,7 +16093,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>44.65%</t>
+          <t>17.93%</t>
         </is>
       </c>
       <c r="J39" t="str">
@@ -16148,7 +16149,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-2.88%</t>
         </is>
       </c>
       <c r="J40" t="str">
@@ -16204,7 +16205,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>70.48%</t>
+          <t>54.29%</t>
         </is>
       </c>
       <c r="J41" t="str">
@@ -16260,7 +16261,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>0.89%</t>
+          <t>-7.06%</t>
         </is>
       </c>
       <c r="J42" t="str">
@@ -16316,7 +16317,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>12.77%</t>
+          <t>-15.78%</t>
         </is>
       </c>
       <c r="J43" t="str">
@@ -16372,7 +16373,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>40.98%</t>
+          <t>9.35%</t>
         </is>
       </c>
       <c r="J44" t="str">
@@ -16542,7 +16543,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>10.81%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="J47" t="str">
@@ -16598,7 +16599,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>30.11%</t>
+          <t>-0.35%</t>
         </is>
       </c>
       <c r="J48" t="str">
@@ -16654,7 +16655,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>8.64%</t>
+          <t>-8.44%</t>
         </is>
       </c>
       <c r="J49" t="str">
@@ -16710,7 +16711,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>12.32%</t>
+          <t>-6.01%</t>
         </is>
       </c>
       <c r="J50" t="str">
@@ -16766,7 +16767,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>15.08%</t>
+          <t>-3.19%</t>
         </is>
       </c>
       <c r="J51" t="str">
@@ -16822,7 +16823,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>-43.80%</t>
+          <t>-47.37%</t>
         </is>
       </c>
       <c r="J52" t="str">
@@ -16992,13 +16993,12 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>-7.94%</t>
+        </is>
+      </c>
+      <c r="J55" t="str">
+        <f>HYPERLINK("kline_charts/BK0963_商业航天.html","打开K线图")</f>
+        <v>打开K线图</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -17049,7 +17049,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>-3.85%</t>
+          <t>-20.41%</t>
         </is>
       </c>
       <c r="J56" t="str">
@@ -17105,7 +17105,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>24.28%</t>
+          <t>9.44%</t>
         </is>
       </c>
       <c r="J57" t="str">
@@ -17161,7 +17161,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>54.27%</t>
+          <t>30.64%</t>
         </is>
       </c>
       <c r="J58" t="str">
@@ -17217,7 +17217,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>25.93%</t>
+          <t>8.26%</t>
         </is>
       </c>
       <c r="J59" t="str">
@@ -17330,7 +17330,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>41.56%</t>
+          <t>27.87%</t>
         </is>
       </c>
       <c r="J61" t="str">
@@ -17386,7 +17386,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>-7.57%</t>
         </is>
       </c>
       <c r="J62" t="str">
@@ -17442,7 +17442,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>85.13%</t>
+          <t>56.69%</t>
         </is>
       </c>
       <c r="J63" t="str">
@@ -17498,7 +17498,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>43.60%</t>
+          <t>16.78%</t>
         </is>
       </c>
       <c r="J64" t="str">
@@ -17554,7 +17554,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>-8.92%</t>
         </is>
       </c>
       <c r="J65" t="str">
@@ -17610,7 +17610,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>37.68%</t>
+          <t>17.54%</t>
         </is>
       </c>
       <c r="J66" t="str">
@@ -17723,7 +17723,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>9.54%</t>
+          <t>2.03%</t>
         </is>
       </c>
       <c r="J68" t="str">
@@ -17779,7 +17779,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>38.30%</t>
+          <t>23.27%</t>
         </is>
       </c>
       <c r="J69" t="str">
@@ -17835,7 +17835,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>11.26%</t>
+          <t>2.24%</t>
         </is>
       </c>
       <c r="J70" t="str">
@@ -17891,7 +17891,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>11.82%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="J71" t="str">
@@ -17947,7 +17947,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>-9.79%</t>
+          <t>-9.52%</t>
         </is>
       </c>
       <c r="J72" t="str">
@@ -18060,7 +18060,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>41.36%</t>
+          <t>20.74%</t>
         </is>
       </c>
       <c r="J74" t="str">
@@ -18116,7 +18116,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>5.27%</t>
+          <t>-12.74%</t>
         </is>
       </c>
       <c r="J75" t="str">
@@ -18172,7 +18172,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>1.93%</t>
+          <t>-11.25%</t>
         </is>
       </c>
       <c r="J76" t="str">
@@ -18228,7 +18228,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>28.39%</t>
+          <t>7.05%</t>
         </is>
       </c>
       <c r="J77" t="str">
@@ -18284,7 +18284,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>28.14%</t>
+          <t>4.10%</t>
         </is>
       </c>
       <c r="J78" t="str">
@@ -18454,7 +18454,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>65.63%</t>
+          <t>51.52%</t>
         </is>
       </c>
       <c r="J81" t="str">
@@ -18510,7 +18510,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>34.35%</t>
+          <t>20.69%</t>
         </is>
       </c>
       <c r="J82" t="str">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>77.86%</t>
+          <t>78.62%</t>
         </is>
       </c>
       <c r="J83" t="str">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>34.24%</t>
+          <t>8.67%</t>
         </is>
       </c>
       <c r="J85" t="str">
@@ -18735,7 +18735,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>64.18%</t>
+          <t>21.03%</t>
         </is>
       </c>
       <c r="J86" t="str">
@@ -18905,7 +18905,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>10.24%</t>
+          <t>-9.50%</t>
         </is>
       </c>
       <c r="J89" t="str">
@@ -19018,7 +19018,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>35.79%</t>
+          <t>10.51%</t>
         </is>
       </c>
       <c r="J91" t="str">
@@ -19074,7 +19074,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>32.52%</t>
+          <t>10.06%</t>
         </is>
       </c>
       <c r="J92" t="str">

</xml_diff>